<commit_message>
ditall updates, 1. version
</commit_message>
<xml_diff>
--- a/Ditall/ditall_sablon.xlsx
+++ b/Ditall/ditall_sablon.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zsomborgalgoczi/Desktop/workspace/github.com/zsombzs/label_generator/Ditall/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA1F38A4-88E2-5541-A2ED-22C0D6F1AA0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2082992F-7F5A-F942-8BBF-C0BCA647E249}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16960" xr2:uid="{195B7CB8-57D0-714D-A057-F87136F4FC09}"/>
   </bookViews>
@@ -53,7 +53,7 @@
     <t>Ár</t>
   </si>
   <si>
-    <t>Akciós_ár</t>
+    <t>Szín</t>
   </si>
 </sst>
 </file>
@@ -90,7 +90,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -102,7 +102,9 @@
       <left style="thick">
         <color auto="1"/>
       </left>
-      <right/>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
       <top style="thick">
         <color auto="1"/>
       </top>
@@ -115,33 +117,7 @@
       <left style="thick">
         <color auto="1"/>
       </left>
-      <right style="thick">
-        <color auto="1"/>
-      </right>
-      <top style="thick">
-        <color auto="1"/>
-      </top>
-      <bottom style="double">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color auto="1"/>
-      </right>
-      <top style="thick">
-        <color auto="1"/>
-      </top>
-      <bottom style="double">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
+      <right style="thin">
         <color auto="1"/>
       </right>
       <top/>
@@ -149,16 +125,18 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thick">
+      <left style="thin">
         <color auto="1"/>
       </left>
-      <right/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thick">
+      <left style="thin">
         <color auto="1"/>
       </left>
       <right style="thick">
@@ -172,26 +150,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -526,208 +495,37 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0807640-E514-5C42-8365-97613778117F}">
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="35.1640625" style="7" customWidth="1"/>
-    <col min="2" max="2" width="29.33203125" customWidth="1"/>
-    <col min="3" max="3" width="33.33203125" customWidth="1"/>
-    <col min="4" max="4" width="27.33203125" customWidth="1"/>
-    <col min="5" max="6" width="29" style="5" customWidth="1"/>
+    <col min="1" max="1" width="33.33203125" style="2" customWidth="1"/>
+    <col min="2" max="4" width="27.33203125" style="3" customWidth="1"/>
+    <col min="5" max="5" width="29" style="3" customWidth="1"/>
+    <col min="6" max="6" width="35.1640625" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="43" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>5</v>
+      <c r="F1" s="1" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="17" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="6"/>
-      <c r="B2" s="4"/>
-      <c r="F2" s="8"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F3" s="8"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F4" s="8"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F5" s="8"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F6" s="8"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F7" s="8"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F8" s="8"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F9" s="8"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F10" s="8"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F11" s="8"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F12" s="8"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F13" s="8"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F14" s="8"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F15" s="8"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F16" s="8"/>
-    </row>
-    <row r="17" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F17" s="8"/>
-    </row>
-    <row r="18" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F18" s="8"/>
-    </row>
-    <row r="19" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F19" s="8"/>
-    </row>
-    <row r="20" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F20" s="8"/>
-    </row>
-    <row r="21" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F21" s="8"/>
-    </row>
-    <row r="22" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F22" s="8"/>
-    </row>
-    <row r="23" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F23" s="8"/>
-    </row>
-    <row r="24" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F24" s="8"/>
-    </row>
-    <row r="25" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F25" s="8"/>
-    </row>
-    <row r="26" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F26" s="8"/>
-    </row>
-    <row r="27" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F27" s="8"/>
-    </row>
-    <row r="28" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F28" s="8"/>
-    </row>
-    <row r="29" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F29" s="8"/>
-    </row>
-    <row r="30" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F30" s="8"/>
-    </row>
-    <row r="31" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F31" s="8"/>
-    </row>
-    <row r="32" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F32" s="8"/>
-    </row>
-    <row r="33" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F33" s="8"/>
-    </row>
-    <row r="34" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F34" s="8"/>
-    </row>
-    <row r="35" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F35" s="8"/>
-    </row>
-    <row r="36" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F36" s="8"/>
-    </row>
-    <row r="37" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F37" s="8"/>
-    </row>
-    <row r="38" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F38" s="8"/>
-    </row>
-    <row r="39" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F39" s="8"/>
-    </row>
-    <row r="40" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F40" s="8"/>
-    </row>
-    <row r="41" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F41" s="8"/>
-    </row>
-    <row r="42" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F42" s="8"/>
-    </row>
-    <row r="43" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F43" s="8"/>
-    </row>
-    <row r="44" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F44" s="8"/>
-    </row>
-    <row r="45" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F45" s="8"/>
-    </row>
-    <row r="46" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F46" s="8"/>
-    </row>
-    <row r="47" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F47" s="8"/>
-    </row>
-    <row r="48" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F48" s="8"/>
-    </row>
-    <row r="49" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F49" s="8"/>
-    </row>
-    <row r="50" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F50" s="8"/>
-    </row>
-    <row r="51" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F51" s="8"/>
-    </row>
-    <row r="52" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F52" s="8"/>
-    </row>
-    <row r="53" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F53" s="8"/>
-    </row>
-    <row r="54" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F54" s="8"/>
-    </row>
-    <row r="55" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F55" s="8"/>
-    </row>
-    <row r="56" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F56" s="8"/>
-    </row>
-    <row r="57" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F57" s="8"/>
-    </row>
-    <row r="58" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F58" s="8"/>
+      <c r="F2" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>